<commit_message>
Preparing to get costs for the maximum water production, summer
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/Cumulative_water_production_figure.xlsx
+++ b/tutorials/flex_ro/sweep results/Cumulative_water_production_figure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49B6836-C423-428F-AB64-113BB2BB9AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3DCE63-BE44-47F9-91A9-39DD004E27ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1" xr2:uid="{7FA62C76-76A4-4D26-9ABE-794AE35D94A5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7FA62C76-76A4-4D26-9ABE-794AE35D94A5}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="1" r:id="rId1"/>
@@ -252,10 +252,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-  </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -277,12 +274,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -317,20 +308,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15385,13 +15375,13 @@
       <c r="Q7">
         <v>8000</v>
       </c>
-      <c r="R7">
+      <c r="R7" s="6">
         <v>188119.78080000001</v>
       </c>
-      <c r="S7" s="8">
+      <c r="S7" s="6">
         <v>201617.2697</v>
       </c>
-      <c r="T7" s="8">
+      <c r="T7" s="6">
         <f>S7-$V$3</f>
         <v>80066.269700000004</v>
       </c>
@@ -15424,13 +15414,13 @@
         <f>AA7*30/7</f>
         <v>343141.14762048423</v>
       </c>
-      <c r="AG7">
+      <c r="AG7" s="6">
         <v>188119.78084509599</v>
       </c>
       <c r="AH7">
         <v>195648.76172563501</v>
       </c>
-      <c r="AI7" s="5">
+      <c r="AI7" s="6">
         <f>AH7-$V$3</f>
         <v>74097.761725635006</v>
       </c>
@@ -15531,13 +15521,13 @@
       <c r="Q8">
         <v>9000</v>
       </c>
-      <c r="R8">
+      <c r="R8" s="6">
         <v>211634.75339999999</v>
       </c>
-      <c r="S8" s="8">
+      <c r="S8" s="6">
         <v>210740.57440000001</v>
       </c>
-      <c r="T8" s="8">
+      <c r="T8" s="6">
         <f t="shared" ref="T8:T14" si="1">S8-$V$3</f>
         <v>89189.574400000012</v>
       </c>
@@ -15570,13 +15560,13 @@
         <f>AA8*30/7</f>
         <v>509698.12750989851</v>
       </c>
-      <c r="AG8">
+      <c r="AG8" s="6">
         <v>236075</v>
       </c>
       <c r="AH8">
         <v>215765.27735091501</v>
       </c>
-      <c r="AI8" s="5">
+      <c r="AI8" s="6">
         <f t="shared" ref="AI8:AI11" si="6">AH8-$V$3</f>
         <v>94214.277350915014</v>
       </c>
@@ -15671,13 +15661,13 @@
       <c r="Q9">
         <v>10000</v>
       </c>
-      <c r="R9">
+      <c r="R9" s="6">
         <v>235149.726</v>
       </c>
-      <c r="S9" s="8">
+      <c r="S9" s="6">
         <v>220205.54380000001</v>
       </c>
-      <c r="T9" s="8">
+      <c r="T9" s="6">
         <f t="shared" si="1"/>
         <v>98654.543800000014</v>
       </c>
@@ -15710,13 +15700,13 @@
         <f>AA9*30/7</f>
         <v>514712.31871507276</v>
       </c>
-      <c r="AG9">
+      <c r="AG9" s="6">
         <v>282179.67125493102</v>
       </c>
       <c r="AH9">
         <v>233294.366687267</v>
       </c>
-      <c r="AI9" s="5">
+      <c r="AI9" s="6">
         <f t="shared" si="6"/>
         <v>111743.366687267</v>
       </c>
@@ -15823,13 +15813,13 @@
       <c r="Q10">
         <v>11000</v>
       </c>
-      <c r="R10">
+      <c r="R10" s="6">
         <v>258665.41560000001</v>
       </c>
-      <c r="S10" s="8">
+      <c r="S10" s="6">
         <v>229216.2788</v>
       </c>
-      <c r="T10" s="8">
+      <c r="T10" s="6">
         <f t="shared" si="1"/>
         <v>107665.2788</v>
       </c>
@@ -15862,13 +15852,13 @@
         <f>AA10*30/7</f>
         <v>680707.86862926849</v>
       </c>
-      <c r="AG10">
+      <c r="AG10" s="6">
         <v>329242.04908676498</v>
       </c>
       <c r="AH10">
         <v>252044.54975234199</v>
       </c>
-      <c r="AI10" s="5">
+      <c r="AI10" s="6">
         <f t="shared" si="6"/>
         <v>130493.54975234199</v>
       </c>
@@ -15972,13 +15962,13 @@
       <c r="Q11">
         <v>12000</v>
       </c>
-      <c r="R11">
+      <c r="R11" s="6">
         <v>282179.67119999998</v>
       </c>
-      <c r="S11" s="8">
+      <c r="S11" s="6">
         <v>239283.03289999999</v>
       </c>
-      <c r="T11" s="8">
+      <c r="T11" s="6">
         <f t="shared" si="1"/>
         <v>117732.03289999999</v>
       </c>
@@ -16008,13 +15998,13 @@
         <f>AA11*30/7</f>
         <v>687622.98458399589</v>
       </c>
-      <c r="AG11">
+      <c r="AG11" s="6">
         <v>376239.56164384098</v>
       </c>
       <c r="AH11">
         <v>272268.28385817702</v>
       </c>
-      <c r="AI11" s="5">
+      <c r="AI11" s="6">
         <f t="shared" si="6"/>
         <v>150717.28385817702</v>
       </c>
@@ -16121,13 +16111,13 @@
       <c r="Q12">
         <v>13000</v>
       </c>
-      <c r="R12">
+      <c r="R12" s="6">
         <v>305694.64380000002</v>
       </c>
-      <c r="S12" s="8">
+      <c r="S12" s="6">
         <v>247634.47459999999</v>
       </c>
-      <c r="T12" s="8">
+      <c r="T12" s="6">
         <f t="shared" si="1"/>
         <v>126083.47459999999</v>
       </c>
@@ -16222,13 +16212,13 @@
       <c r="Q13">
         <v>14000</v>
       </c>
-      <c r="R13">
+      <c r="R13" s="6">
         <v>329281.85550000001</v>
       </c>
-      <c r="S13" s="8">
+      <c r="S13" s="6">
         <v>257639.08540000001</v>
       </c>
-      <c r="T13" s="8">
+      <c r="T13" s="6">
         <f t="shared" si="1"/>
         <v>136088.08540000001</v>
       </c>
@@ -16335,13 +16325,13 @@
       <c r="Q14">
         <v>15000</v>
       </c>
-      <c r="R14">
+      <c r="R14" s="6">
         <v>352724.58906158298</v>
       </c>
-      <c r="S14" s="8">
+      <c r="S14" s="6">
         <v>267783.90667359199</v>
       </c>
-      <c r="T14" s="8">
+      <c r="T14" s="6">
         <f t="shared" si="1"/>
         <v>146232.90667359199</v>
       </c>
@@ -16445,13 +16435,13 @@
       <c r="Q15">
         <v>16000</v>
       </c>
-      <c r="R15">
+      <c r="R15" s="6">
         <v>376241.59049999999</v>
       </c>
-      <c r="S15" s="8">
+      <c r="S15" s="6">
         <v>280887.32260000001</v>
       </c>
-      <c r="T15" s="8">
+      <c r="T15" s="6">
         <f>S15-$V$3</f>
         <v>159336.32260000001</v>
       </c>
@@ -16845,7 +16835,7 @@
       <c r="T57" s="7"/>
       <c r="U57" s="7"/>
       <c r="V57" s="7"/>
-      <c r="W57" s="6"/>
+      <c r="W57" s="5"/>
     </row>
     <row r="58" spans="17:23" x14ac:dyDescent="0.4">
       <c r="S58" s="7" t="s">
@@ -16856,7 +16846,7 @@
         <v>39</v>
       </c>
       <c r="V58" s="7"/>
-      <c r="W58" s="6"/>
+      <c r="W58" s="5"/>
     </row>
     <row r="59" spans="17:23" x14ac:dyDescent="0.4">
       <c r="Q59" t="s">
@@ -17084,8 +17074,9 @@
     <mergeCell ref="U58:V58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Moving around water sweep files
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/Cumulative_water_production_figure.xlsx
+++ b/tutorials/flex_ro/sweep results/Cumulative_water_production_figure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3DCE63-BE44-47F9-91A9-39DD004E27ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E9062CC-C546-4B6B-9150-C0EA8778CB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7FA62C76-76A4-4D26-9ABE-794AE35D94A5}"/>
   </bookViews>
@@ -14005,12 +14005,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FD001A-7560-4528-B9C4-403F98F24F29}">
   <dimension ref="B2:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="23.84375" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:28" x14ac:dyDescent="0.35">
       <c r="C2" s="7" t="s">
         <v>19</v>
       </c>
@@ -14041,7 +14041,7 @@
       <c r="AA2" s="7"/>
       <c r="AB2" s="7"/>
     </row>
-    <row r="4" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:28" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>1</v>
       </c>
@@ -14115,7 +14115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -14213,7 +14213,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>15</v>
       </c>
@@ -14293,7 +14293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>4</v>
       </c>
@@ -14397,7 +14397,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>16</v>
       </c>
@@ -14477,7 +14477,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>4</v>
       </c>
@@ -14581,7 +14581,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>5</v>
       </c>
@@ -14661,7 +14661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>4</v>
       </c>
@@ -14765,7 +14765,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="12" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>17</v>
       </c>
@@ -14845,7 +14845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>4</v>
       </c>
@@ -14949,7 +14949,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="14" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>18</v>
       </c>
@@ -15029,7 +15029,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="2:28" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:28" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>4</v>
       </c>
@@ -15147,23 +15147,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C55A24DE-0357-403E-9E88-9808FEC167BA}">
   <dimension ref="B3:BA68"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="16.3828125" customWidth="1"/>
-    <col min="16" max="16" width="3.07421875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="10.23046875" customWidth="1"/>
-    <col min="19" max="19" width="14.3828125" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" customWidth="1"/>
+    <col min="16" max="16" width="3.08984375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="10.26953125" customWidth="1"/>
+    <col min="19" max="19" width="14.36328125" customWidth="1"/>
     <col min="20" max="21" width="14" customWidth="1"/>
-    <col min="29" max="29" width="14.15234375" customWidth="1"/>
-    <col min="33" max="33" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.84375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.15234375" customWidth="1"/>
-    <col min="36" max="36" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.84375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="5.23046875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" customWidth="1"/>
+    <col min="33" max="33" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.1796875" customWidth="1"/>
+    <col min="36" max="36" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="5.26953125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:53" x14ac:dyDescent="0.35">
       <c r="U3" s="2" t="s">
         <v>26</v>
       </c>
@@ -15174,12 +15174,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:53" x14ac:dyDescent="0.35">
       <c r="S4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:53" x14ac:dyDescent="0.35">
       <c r="C5" s="7" t="s">
         <v>34</v>
       </c>
@@ -15243,7 +15243,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:53" x14ac:dyDescent="0.35">
       <c r="Q6" t="s">
         <v>42</v>
       </c>
@@ -15332,7 +15332,7 @@
         <v>0.89694148746272895</v>
       </c>
     </row>
-    <row r="7" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>0</v>
       </c>
@@ -15472,7 +15472,7 @@
         <v>0.896941487237917</v>
       </c>
     </row>
-    <row r="8" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:53" x14ac:dyDescent="0.35">
       <c r="C8">
         <v>1</v>
       </c>
@@ -15618,7 +15618,7 @@
         <v>0.89694146817453502</v>
       </c>
     </row>
-    <row r="9" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>21</v>
       </c>
@@ -15758,7 +15758,7 @@
         <v>0.89694148704607501</v>
       </c>
     </row>
-    <row r="10" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>28</v>
       </c>
@@ -15910,7 +15910,7 @@
         <v>0.896941485027969</v>
       </c>
     </row>
-    <row r="11" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>27</v>
       </c>
@@ -16056,7 +16056,7 @@
         <v>0.88560670019780996</v>
       </c>
     </row>
-    <row r="12" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>29</v>
       </c>
@@ -16169,7 +16169,7 @@
         <v>0.80749408745858198</v>
       </c>
     </row>
-    <row r="13" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -16270,7 +16270,7 @@
         <v>0.82590429693763701</v>
       </c>
     </row>
-    <row r="14" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>30</v>
       </c>
@@ -16383,7 +16383,7 @@
         <v>0.82222131805057197</v>
       </c>
     </row>
-    <row r="15" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>27</v>
       </c>
@@ -16493,7 +16493,7 @@
         <v>0.81483195386818397</v>
       </c>
     </row>
-    <row r="16" spans="2:53" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:53" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>29</v>
       </c>
@@ -16585,7 +16585,7 @@
         <v>0.811520130866204</v>
       </c>
     </row>
-    <row r="17" spans="25:53" x14ac:dyDescent="0.4">
+    <row r="17" spans="25:53" x14ac:dyDescent="0.35">
       <c r="AO17">
         <v>13000</v>
       </c>
@@ -16626,12 +16626,12 @@
         <v>0.81164660730883198</v>
       </c>
     </row>
-    <row r="31" spans="25:53" x14ac:dyDescent="0.4">
+    <row r="31" spans="25:53" x14ac:dyDescent="0.35">
       <c r="Z31" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="25:53" x14ac:dyDescent="0.4">
+    <row r="32" spans="25:53" x14ac:dyDescent="0.35">
       <c r="Y32" t="s">
         <v>37</v>
       </c>
@@ -16648,7 +16648,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="33" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y33">
         <v>188119.78080000001</v>
       </c>
@@ -16668,7 +16668,7 @@
         <v>343141.15542857145</v>
       </c>
     </row>
-    <row r="34" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="34" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y34">
         <v>211634.75342467701</v>
       </c>
@@ -16688,7 +16688,7 @@
         <v>386579.3856949886</v>
       </c>
     </row>
-    <row r="35" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="35" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y35">
         <v>235150.71465123599</v>
       </c>
@@ -16708,7 +16708,7 @@
         <v>424651.4097304329</v>
       </c>
     </row>
-    <row r="36" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="36" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y36">
         <v>258664.69865969699</v>
       </c>
@@ -16728,7 +16728,7 @@
         <v>473383.28362189711</v>
       </c>
     </row>
-    <row r="37" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="37" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y37">
         <v>282179.67129999999</v>
       </c>
@@ -16748,7 +16748,7 @@
         <v>518160.71828571422</v>
       </c>
     </row>
-    <row r="38" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="38" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y38">
         <v>305900</v>
       </c>
@@ -16768,7 +16768,7 @@
         <v>561827.67614238441</v>
       </c>
     </row>
-    <row r="39" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="39" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y39">
         <v>329209.61660000001</v>
       </c>
@@ -16788,7 +16788,7 @@
         <v>601366.87885714299</v>
       </c>
     </row>
-    <row r="40" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="40" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y40">
         <v>352724.58906469098</v>
       </c>
@@ -16808,7 +16808,7 @@
         <v>643552.06847316015</v>
       </c>
     </row>
-    <row r="41" spans="25:29" x14ac:dyDescent="0.4">
+    <row r="41" spans="25:29" x14ac:dyDescent="0.35">
       <c r="Y41">
         <v>376239.56170000002</v>
       </c>
@@ -16828,7 +16828,7 @@
         <v>687623.00742857135</v>
       </c>
     </row>
-    <row r="57" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="57" spans="17:23" x14ac:dyDescent="0.35">
       <c r="S57" s="7" t="s">
         <v>40</v>
       </c>
@@ -16837,7 +16837,7 @@
       <c r="V57" s="7"/>
       <c r="W57" s="5"/>
     </row>
-    <row r="58" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="58" spans="17:23" x14ac:dyDescent="0.35">
       <c r="S58" s="7" t="s">
         <v>33</v>
       </c>
@@ -16848,7 +16848,7 @@
       <c r="V58" s="7"/>
       <c r="W58" s="5"/>
     </row>
-    <row r="59" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="59" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q59" t="s">
         <v>23</v>
       </c>
@@ -16868,7 +16868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="60" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q60">
         <v>653.60975435751936</v>
       </c>
@@ -16890,7 +16890,7 @@
         <v>99009.749455198325</v>
       </c>
     </row>
-    <row r="61" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="61" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q61">
         <v>735.31097365220921</v>
       </c>
@@ -16912,7 +16912,7 @@
         <v>111346.66422926786</v>
       </c>
     </row>
-    <row r="62" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="62" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q62">
         <v>817.01219294689895</v>
       </c>
@@ -16934,7 +16934,7 @@
         <v>124309.79780110029</v>
       </c>
     </row>
-    <row r="63" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="63" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q63">
         <v>898.71590341073602</v>
       </c>
@@ -16956,7 +16956,7 @@
         <v>132954.54405867599</v>
       </c>
     </row>
-    <row r="64" spans="17:23" x14ac:dyDescent="0.4">
+    <row r="64" spans="17:23" x14ac:dyDescent="0.35">
       <c r="Q64">
         <v>980.41463153627888</v>
       </c>
@@ -16978,7 +16978,7 @@
         <v>151965.71857084543</v>
       </c>
     </row>
-    <row r="65" spans="17:22" x14ac:dyDescent="0.4">
+    <row r="65" spans="17:22" x14ac:dyDescent="0.35">
       <c r="Q65">
         <v>1062.1158508309688</v>
       </c>
@@ -17000,7 +17000,7 @@
         <v>153228.46531289187</v>
       </c>
     </row>
-    <row r="66" spans="17:22" x14ac:dyDescent="0.4">
+    <row r="66" spans="17:22" x14ac:dyDescent="0.35">
       <c r="Q66">
         <v>1144.0680601077077</v>
       </c>
@@ -17022,7 +17022,7 @@
         <v>164270.90201764583</v>
       </c>
     </row>
-    <row r="67" spans="17:22" x14ac:dyDescent="0.4">
+    <row r="67" spans="17:22" x14ac:dyDescent="0.35">
       <c r="Q67">
         <v>1225.5182896343147</v>
       </c>
@@ -17044,7 +17044,7 @@
         <v>181244.68161428574</v>
       </c>
     </row>
-    <row r="68" spans="17:22" x14ac:dyDescent="0.4">
+    <row r="68" spans="17:22" x14ac:dyDescent="0.35">
       <c r="Q68">
         <v>1307.2265579940936</v>
       </c>

</xml_diff>